<commit_message>
Level 1 and 2 Setup, Sweat Particles
</commit_message>
<xml_diff>
--- a/Assets/Resources/ASKFirstDialogue2Options.xlsx
+++ b/Assets/Resources/ASKFirstDialogue2Options.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jayso\ASKFirst v2\Assets\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B3C0C0-CCD5-4746-94DE-4923BE5CCB54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CC93B8-5D09-44C0-B1B4-C5ED0F6A74BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{8CF9D31E-0312-48F0-ADC3-94BF3514D222}"/>
+    <workbookView xWindow="28680" yWindow="-2925" windowWidth="38640" windowHeight="21120" xr2:uid="{8CF9D31E-0312-48F0-ADC3-94BF3514D222}"/>
   </bookViews>
   <sheets>
     <sheet name="ASKFirstDialogue2Options" sheetId="1" r:id="rId1"/>
@@ -1148,12 +1148,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F60FC667-4F56-45C1-A2CA-D070B5A8D91D}">
   <dimension ref="A1:U58"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="22" width="40.7265625" customWidth="1"/>
+    <col min="1" max="22" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1307,7 +1307,7 @@
       <c r="N3" s="1"/>
       <c r="R3" s="1"/>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1331,7 +1331,7 @@
       <c r="N4" s="1"/>
       <c r="R4" s="1"/>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1396,7 +1396,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1420,7 +1420,7 @@
       <c r="N6" s="1"/>
       <c r="R6" s="1"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -1444,7 +1444,7 @@
       <c r="N7" s="1"/>
       <c r="R7" s="1"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>35</v>
       </c>
@@ -1509,7 +1509,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -1533,7 +1533,7 @@
       <c r="N9" s="1"/>
       <c r="R9" s="1"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -1557,7 +1557,7 @@
       <c r="N10" s="1"/>
       <c r="R10" s="1"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>35</v>
       </c>
@@ -1581,7 +1581,7 @@
       <c r="N11" s="1"/>
       <c r="R11" s="1"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -1608,7 +1608,7 @@
       <c r="N12" s="1"/>
       <c r="R12" s="1"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>45</v>
       </c>
@@ -1651,7 +1651,7 @@
       <c r="N13" s="1"/>
       <c r="R13" s="1"/>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -1675,7 +1675,7 @@
       <c r="N14" s="1"/>
       <c r="R14" s="1"/>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>45</v>
       </c>
@@ -1699,7 +1699,7 @@
       <c r="N15" s="1"/>
       <c r="R15" s="1"/>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>45</v>
       </c>
@@ -1723,7 +1723,7 @@
       <c r="N16" s="1"/>
       <c r="R16" s="1"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>50</v>
       </c>
@@ -1748,11 +1748,14 @@
       <c r="H17">
         <v>-3</v>
       </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
       <c r="J17" s="1" t="s">
         <v>52</v>
       </c>
       <c r="K17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L17">
         <v>2</v>
@@ -1763,7 +1766,7 @@
       <c r="N17" s="1"/>
       <c r="R17" s="1"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>50</v>
       </c>
@@ -1788,6 +1791,9 @@
       <c r="H18">
         <v>-7</v>
       </c>
+      <c r="I18">
+        <v>4</v>
+      </c>
       <c r="J18" s="1" t="s">
         <v>57</v>
       </c>
@@ -1797,10 +1803,13 @@
       <c r="L18">
         <v>3</v>
       </c>
+      <c r="M18">
+        <v>5</v>
+      </c>
       <c r="N18" s="1"/>
       <c r="R18" s="1"/>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>50</v>
       </c>
@@ -1824,7 +1833,7 @@
       <c r="N19" s="1"/>
       <c r="R19" s="1"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>50</v>
       </c>
@@ -1848,7 +1857,7 @@
       <c r="N20" s="1"/>
       <c r="R20" s="1"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>50</v>
       </c>
@@ -1872,7 +1881,7 @@
       <c r="N21" s="1"/>
       <c r="R21" s="1"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>60</v>
       </c>
@@ -1912,7 +1921,7 @@
       <c r="N22" s="1"/>
       <c r="R22" s="1"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>60</v>
       </c>
@@ -1949,7 +1958,7 @@
       <c r="N23" s="1"/>
       <c r="R23" s="1"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>60</v>
       </c>
@@ -1973,7 +1982,7 @@
       <c r="N24" s="1"/>
       <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>60</v>
       </c>
@@ -1997,7 +2006,7 @@
       <c r="N25" s="1"/>
       <c r="R25" s="1"/>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>60</v>
       </c>
@@ -2021,7 +2030,7 @@
       <c r="N26" s="1"/>
       <c r="R26" s="1"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>70</v>
       </c>
@@ -2058,7 +2067,7 @@
       <c r="N27" s="1"/>
       <c r="R27" s="1"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>70</v>
       </c>
@@ -2095,7 +2104,7 @@
       <c r="N28" s="1"/>
       <c r="R28" s="1"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>70</v>
       </c>
@@ -2119,7 +2128,7 @@
       <c r="N29" s="1"/>
       <c r="R29" s="1"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>70</v>
       </c>
@@ -2156,7 +2165,7 @@
       <c r="N30" s="1"/>
       <c r="R30" s="1"/>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>70</v>
       </c>
@@ -2180,7 +2189,7 @@
       <c r="N31" s="1"/>
       <c r="R31" s="1"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>70</v>
       </c>
@@ -2204,182 +2213,182 @@
       <c r="N32" s="1"/>
       <c r="R32" s="1"/>
     </row>
-    <row r="33" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="33" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D33" s="1"/>
       <c r="F33" s="1"/>
       <c r="J33" s="1"/>
       <c r="N33" s="1"/>
       <c r="R33" s="1"/>
     </row>
-    <row r="34" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="34" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D34" s="1"/>
       <c r="F34" s="1"/>
       <c r="J34" s="1"/>
       <c r="N34" s="1"/>
       <c r="R34" s="1"/>
     </row>
-    <row r="35" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="35" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D35" s="1"/>
       <c r="F35" s="1"/>
       <c r="J35" s="1"/>
       <c r="N35" s="1"/>
       <c r="R35" s="1"/>
     </row>
-    <row r="36" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="36" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D36" s="1"/>
       <c r="F36" s="1"/>
       <c r="J36" s="1"/>
       <c r="N36" s="1"/>
       <c r="R36" s="1"/>
     </row>
-    <row r="37" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="37" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D37" s="1"/>
       <c r="F37" s="1"/>
       <c r="J37" s="1"/>
       <c r="N37" s="1"/>
       <c r="R37" s="1"/>
     </row>
-    <row r="38" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="38" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D38" s="1"/>
       <c r="F38" s="1"/>
       <c r="J38" s="1"/>
       <c r="N38" s="1"/>
       <c r="R38" s="1"/>
     </row>
-    <row r="39" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="39" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D39" s="1"/>
       <c r="F39" s="1"/>
       <c r="J39" s="1"/>
       <c r="N39" s="1"/>
       <c r="R39" s="1"/>
     </row>
-    <row r="40" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="40" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D40" s="1"/>
       <c r="F40" s="1"/>
       <c r="J40" s="1"/>
       <c r="N40" s="1"/>
       <c r="R40" s="1"/>
     </row>
-    <row r="41" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="41" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D41" s="1"/>
       <c r="F41" s="1"/>
       <c r="J41" s="1"/>
       <c r="N41" s="1"/>
       <c r="R41" s="1"/>
     </row>
-    <row r="42" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="42" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D42" s="1"/>
       <c r="F42" s="1"/>
       <c r="J42" s="1"/>
       <c r="N42" s="1"/>
       <c r="R42" s="1"/>
     </row>
-    <row r="43" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="43" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D43" s="1"/>
       <c r="F43" s="1"/>
       <c r="J43" s="1"/>
       <c r="N43" s="1"/>
       <c r="R43" s="1"/>
     </row>
-    <row r="44" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="44" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D44" s="1"/>
       <c r="F44" s="1"/>
       <c r="J44" s="1"/>
       <c r="N44" s="1"/>
       <c r="R44" s="1"/>
     </row>
-    <row r="45" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="45" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D45" s="1"/>
       <c r="F45" s="1"/>
       <c r="J45" s="1"/>
       <c r="N45" s="1"/>
       <c r="R45" s="1"/>
     </row>
-    <row r="46" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="46" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D46" s="1"/>
       <c r="F46" s="1"/>
       <c r="J46" s="1"/>
       <c r="N46" s="1"/>
       <c r="R46" s="1"/>
     </row>
-    <row r="47" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="47" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D47" s="1"/>
       <c r="F47" s="1"/>
       <c r="J47" s="1"/>
       <c r="N47" s="1"/>
       <c r="R47" s="1"/>
     </row>
-    <row r="48" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="48" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D48" s="1"/>
       <c r="F48" s="1"/>
       <c r="J48" s="1"/>
       <c r="N48" s="1"/>
       <c r="R48" s="1"/>
     </row>
-    <row r="49" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="49" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D49" s="1"/>
       <c r="F49" s="1"/>
       <c r="J49" s="1"/>
       <c r="N49" s="1"/>
       <c r="R49" s="1"/>
     </row>
-    <row r="50" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="50" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D50" s="1"/>
       <c r="F50" s="1"/>
       <c r="J50" s="1"/>
       <c r="N50" s="1"/>
       <c r="R50" s="1"/>
     </row>
-    <row r="51" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="51" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D51" s="1"/>
       <c r="F51" s="1"/>
       <c r="J51" s="1"/>
       <c r="N51" s="1"/>
       <c r="R51" s="1"/>
     </row>
-    <row r="52" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="52" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D52" s="1"/>
       <c r="F52" s="1"/>
       <c r="J52" s="1"/>
       <c r="N52" s="1"/>
       <c r="R52" s="1"/>
     </row>
-    <row r="53" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="53" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D53" s="1"/>
       <c r="F53" s="1"/>
       <c r="J53" s="1"/>
       <c r="N53" s="1"/>
       <c r="R53" s="1"/>
     </row>
-    <row r="54" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="54" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D54" s="1"/>
       <c r="F54" s="1"/>
       <c r="J54" s="1"/>
       <c r="N54" s="1"/>
       <c r="R54" s="1"/>
     </row>
-    <row r="55" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="55" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D55" s="1"/>
       <c r="F55" s="1"/>
       <c r="J55" s="1"/>
       <c r="N55" s="1"/>
       <c r="R55" s="1"/>
     </row>
-    <row r="56" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="56" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D56" s="1"/>
       <c r="F56" s="1"/>
       <c r="J56" s="1"/>
       <c r="N56" s="1"/>
       <c r="R56" s="1"/>
     </row>
-    <row r="57" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="57" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D57" s="1"/>
       <c r="F57" s="1"/>
       <c r="J57" s="1"/>
       <c r="N57" s="1"/>
       <c r="R57" s="1"/>
     </row>
-    <row r="58" spans="4:18" x14ac:dyDescent="0.35">
+    <row r="58" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D58" s="1"/>
       <c r="F58" s="1"/>
       <c r="J58" s="1"/>

</xml_diff>